<commit_message>
Reorganize prompts into topic folders; add dossier figures for recruitment-hiring, SLA/HR-IT, interpreter regulation, neurodivergence, and outsourced services batches
Moves flat prompt files under prompts/ into per-topic subfolders
(AIS, ATW-PIP, BSL-Act, CODA, Chinese-Walls, DAGM, and others) and
archives superseded master files under prompts/_master-and-misc/.
Adds verified dossier figures for the access-to-work domain and
other batches researched this session, plus prompt 170 verifying
the Murphy v Sheffield Hallam University primary transcript.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EBzVShtsyLreHuwvHDtYLG
</commit_message>
<xml_diff>
--- a/foi-tracking/BSL-FOI-companion-log.xlsx
+++ b/foi-tracking/BSL-FOI-companion-log.xlsx
@@ -3358,7 +3358,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:C20"/>
+  <dimension ref="B2:C20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -3366,7 +3366,6 @@
     <col width="88" customWidth="1" style="73" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="25.5" customHeight="1" s="74">
       <c r="B2" s="88" t="inlineStr">
         <is>
@@ -3381,7 +3380,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="19.5" customHeight="1" s="74">
       <c r="B5" s="101" t="inlineStr">
         <is>
@@ -3452,7 +3450,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="36" customHeight="1" s="74">
       <c r="B12" s="104" t="inlineStr">
         <is>
@@ -3465,7 +3462,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="74">
       <c r="B14" s="78" t="inlineStr">
         <is>
@@ -3540,7 +3536,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="27.75" customHeight="1" s="74">
       <c r="B20" s="109" t="inlineStr">
         <is>
@@ -3575,7 +3570,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:C20"/>
+  <dimension ref="B2:C20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -3583,7 +3578,6 @@
     <col width="88" customWidth="1" style="73" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="25.5" customHeight="1" s="74">
       <c r="B2" s="88" t="inlineStr">
         <is>
@@ -3598,7 +3592,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="19.5" customHeight="1" s="74">
       <c r="B5" s="101" t="inlineStr">
         <is>
@@ -3669,7 +3662,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="36" customHeight="1" s="74">
       <c r="B12" s="104" t="inlineStr">
         <is>
@@ -3682,7 +3674,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="74">
       <c r="B14" s="78" t="inlineStr">
         <is>
@@ -3757,7 +3748,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="27.75" customHeight="1" s="74">
       <c r="B20" s="109" t="inlineStr">
         <is>
@@ -3792,7 +3782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:C20"/>
+  <dimension ref="B2:C20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -3800,7 +3790,6 @@
     <col width="88" customWidth="1" style="73" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="25.5" customHeight="1" s="74">
       <c r="B2" s="88" t="inlineStr">
         <is>
@@ -3815,7 +3804,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="19.5" customHeight="1" s="74">
       <c r="B5" s="101" t="inlineStr">
         <is>
@@ -3886,7 +3874,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="36" customHeight="1" s="74">
       <c r="B12" s="104" t="inlineStr">
         <is>
@@ -3899,7 +3886,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="74">
       <c r="B14" s="78" t="inlineStr">
         <is>
@@ -3973,7 +3959,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="27.75" customHeight="1" s="74">
       <c r="B20" s="109" t="inlineStr">
         <is>
@@ -4008,7 +3993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:C20"/>
+  <dimension ref="B2:C20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -4016,7 +4001,6 @@
     <col width="88" customWidth="1" style="73" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="25.5" customHeight="1" s="74">
       <c r="B2" s="88" t="inlineStr">
         <is>
@@ -4031,7 +4015,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="19.5" customHeight="1" s="74">
       <c r="B5" s="101" t="inlineStr">
         <is>
@@ -4102,7 +4085,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="36" customHeight="1" s="74">
       <c r="B12" s="104" t="inlineStr">
         <is>
@@ -4115,7 +4097,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="74">
       <c r="B14" s="78" t="inlineStr">
         <is>
@@ -4189,7 +4170,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="27.75" customHeight="1" s="74">
       <c r="B20" s="109" t="inlineStr">
         <is>
@@ -4224,7 +4204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:C20"/>
+  <dimension ref="B2:C20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -4232,7 +4212,6 @@
     <col width="88" customWidth="1" style="73" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="25.5" customHeight="1" s="74">
       <c r="B2" s="88" t="inlineStr">
         <is>
@@ -4247,7 +4226,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="19.5" customHeight="1" s="74">
       <c r="B5" s="101" t="inlineStr">
         <is>
@@ -4318,7 +4296,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="36" customHeight="1" s="74">
       <c r="B12" s="104" t="inlineStr">
         <is>
@@ -4331,7 +4308,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="74">
       <c r="B14" s="78" t="inlineStr">
         <is>
@@ -4406,7 +4382,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="27.75" customHeight="1" s="74">
       <c r="B20" s="109" t="inlineStr">
         <is>
@@ -4441,7 +4416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:C20"/>
+  <dimension ref="B2:C20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="3" customWidth="1" style="73" min="1" max="1"/>
@@ -4449,7 +4424,6 @@
     <col width="88" customWidth="1" style="73" min="3" max="3"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="25.5" customHeight="1" s="74">
       <c r="B2" s="88" t="inlineStr">
         <is>
@@ -4464,7 +4438,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5" ht="19.5" customHeight="1" s="74">
       <c r="B5" s="101" t="inlineStr">
         <is>
@@ -4535,7 +4508,6 @@
         </is>
       </c>
     </row>
-    <row r="11"/>
     <row r="12" ht="36" customHeight="1" s="74">
       <c r="B12" s="104" t="inlineStr">
         <is>
@@ -4548,7 +4520,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14" ht="15" customHeight="1" s="74">
       <c r="B14" s="78" t="inlineStr">
         <is>
@@ -4619,7 +4590,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20" ht="27.75" customHeight="1" s="74">
       <c r="B20" s="109" t="inlineStr">
         <is>
@@ -6726,12 +6696,127 @@
       <c r="R40" s="102" t="n"/>
       <c r="S40" s="112" t="n"/>
     </row>
+    <row r="41">
+      <c r="A41" s="111" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="102" t="n"/>
+      <c r="C41" s="102" t="inlineStr">
+        <is>
+          <t>SWL ICB constituent Trusts</t>
+        </is>
+      </c>
+      <c r="D41" s="102" t="inlineStr">
+        <is>
+          <t>Trust</t>
+        </is>
+      </c>
+      <c r="E41" s="102" t="inlineStr">
+        <is>
+          <t>Count of AIS-flagged patients contacted by phone instead of recorded accessible method, and planned appointments where VRI was used/offered instead of a booked in-person BSL interpreter, last 24 months</t>
+        </is>
+      </c>
+      <c r="F41" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="G41" s="114" t="n"/>
+      <c r="H41" s="115">
+        <f>IF(G41="","",WORKDAY(G41,20,$U$5:$U$28))</f>
+        <v/>
+      </c>
+      <c r="I41" s="116">
+        <f>IF(H41="","",H41-TODAY())</f>
+        <v/>
+      </c>
+      <c r="J41" s="114" t="n"/>
+      <c r="K41" s="102" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L41" s="102" t="n"/>
+      <c r="M41" s="102" t="n"/>
+      <c r="N41" s="102" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O41" s="102" t="n"/>
+      <c r="P41" s="102" t="n"/>
+      <c r="Q41" s="102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R41" s="102" t="inlineStr">
+        <is>
+          <t>From AIS prompts 34-37 (8 Sep 2026). Template left blank - closest existing template is T2 (hospital trust activity) but T2 asks about interpreter fulfilment, not contact-method/channel-substitution as its own incident type - expect a "we do not hold this as a reportable field" response, which is itself the finding per the domain briefing. See BSL_DOMAIN_NHS_interpreter_provision.md new subsection and dossier FOI item n:51.</t>
+        </is>
+      </c>
+      <c r="S41" s="112" t="n"/>
+    </row>
     <row r="42" ht="15.75" customHeight="1" s="74">
-      <c r="A42" s="97" t="inlineStr">
-        <is>
-          <t>Counts (auto)</t>
-        </is>
-      </c>
+      <c r="A42" s="111" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="102" t="n"/>
+      <c r="C42" s="102" t="inlineStr">
+        <is>
+          <t>Care Quality Commission (CQC)</t>
+        </is>
+      </c>
+      <c r="D42" s="102" t="inlineStr">
+        <is>
+          <t>Regulator</t>
+        </is>
+      </c>
+      <c r="E42" s="102" t="inlineStr">
+        <is>
+          <t>Whether CQC has ever issued an enforcement notice, fixed penalty, or published inspection finding specifically categorised as an Accessible Information Standard breach (as opposed to a consent/dignity/person-centred-care breach where AIS/BSL is the underlying fact pattern, e.g. UHB "Mr X")</t>
+        </is>
+      </c>
+      <c r="F42" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
+      <c r="G42" s="114" t="n"/>
+      <c r="H42" s="115">
+        <f>IF(G42="","",WORKDAY(G42,20,$U$5:$U$28))</f>
+        <v/>
+      </c>
+      <c r="I42" s="116">
+        <f>IF(H42="","",H42-TODAY())</f>
+        <v/>
+      </c>
+      <c r="J42" s="114" t="n"/>
+      <c r="K42" s="102" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L42" s="102" t="n"/>
+      <c r="M42" s="102" t="n"/>
+      <c r="N42" s="102" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="O42" s="102" t="n"/>
+      <c r="P42" s="102" t="n"/>
+      <c r="Q42" s="102" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="R42" s="102" t="inlineStr">
+        <is>
+          <t>Template left blank - CQC is a regulator, not an ICB/trust/council, so none of T1-T6 apply. From AIS prompt 34 (8 Sep 2026). Tests whether "AIS breach" is a real enforcement category at all - see dossier FOI item n:52 and domain briefing.</t>
+        </is>
+      </c>
+      <c r="S42" s="112" t="n"/>
     </row>
     <row r="43" ht="23.25" customHeight="1" s="74">
       <c r="A43" s="118" t="inlineStr">
@@ -6795,14 +6880,13 @@
         </is>
       </c>
       <c r="B48" s="124">
-        <f>COUNTA(C5:C40)</f>
+        <f>COUNTA(C5:C42)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <autoFilter ref="A4:R60"/>
-  <mergeCells count="3">
-    <mergeCell ref="A42:C42"/>
+  <mergeCells count="2">
     <mergeCell ref="A2:R2"/>
     <mergeCell ref="A1:R1"/>
   </mergeCells>
@@ -6818,27 +6902,27 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="6">
-    <dataValidation sqref="F5:F40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="F5:F42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Not sent,Sent,Due soon,Overdue,Answered — data,Answered — not held,Answered — refused,Internal review,Closed"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="K5:K40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="K5:K42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"—,Full data,Partial data,Not held centrally,Section 12 cost,Section 40 personal data,Section 21 already published,Withdrawn,Internal review"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="N5:N40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="N5:N42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"—,Borough / locality split,Trust-wide only,ICB-wide only,Not held,Suppressed small numbers"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="Q5:Q40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="Q5:Q42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"No,Yes — send T6,Yes — ask named contractor,Yes — internal review,Yes — ask a trust instead"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="B5:B40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="B5:B42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"T1,T2,T3,T4,T5,T6"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation sqref="S5:S40" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
+    <dataValidation sqref="S5:S42" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Add 16 FOI request rows to BSL companion log for the new dossier targets (n:53-67)
Mirrors the FOI targets added to dossier/bsl_dossier.html's DEFAULT_FOI
array in the prior commit, so the tracker and the public dossier stay in
sync. Uses the log's existing pre-numbered blank rows (IDs 17-32);
VRS and EOL-Palliative logs unchanged as none of these targets are
VRS/telecoms or end-of-life specific.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EBzVShtsyLreHuwvHDtYLG
</commit_message>
<xml_diff>
--- a/foi-tracking/BSL-FOI-companion-log.xlsx
+++ b/foi-tracking/BSL-FOI-companion-log.xlsx
@@ -5857,10 +5857,26 @@
         <v>17</v>
       </c>
       <c r="B21" s="102" t="n"/>
-      <c r="C21" s="102" t="n"/>
-      <c r="D21" s="102" t="n"/>
-      <c r="E21" s="102" t="n"/>
-      <c r="F21" s="102" t="n"/>
+      <c r="C21" s="102" t="inlineStr">
+        <is>
+          <t>Department for Work and Pensions (Access to Work)</t>
+        </is>
+      </c>
+      <c r="D21" s="102" t="inlineStr">
+        <is>
+          <t>DWP</t>
+        </is>
+      </c>
+      <c r="E21" s="102" t="inlineStr">
+        <is>
+          <t>Whether the booker/payer identity for AtW-funded interpreting (employer, AtW grant to employee, or agency) is recorded as a discrete field, plus booking/no-show/cancellation counts split by that field, last 12 months.</t>
+        </is>
+      </c>
+      <c r="F21" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G21" s="114" t="n"/>
       <c r="H21" s="115">
         <f>IF(G21="","",WORKDAY(G21,20,$U$5:$U$28))</f>
@@ -5890,8 +5906,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R21" s="102" t="n"/>
-      <c r="S21" s="112" t="n"/>
+      <c r="R21" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:53 (recruitment-hiring batch) — fold into existing log, not a new tracker.</t>
+        </is>
+      </c>
+      <c r="S21" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U21" s="117" t="n">
         <v>46388</v>
       </c>
@@ -5901,10 +5925,26 @@
         <v>18</v>
       </c>
       <c r="B22" s="102" t="n"/>
-      <c r="C22" s="102" t="n"/>
-      <c r="D22" s="102" t="n"/>
-      <c r="E22" s="102" t="n"/>
-      <c r="F22" s="102" t="n"/>
+      <c r="C22" s="102" t="inlineStr">
+        <is>
+          <t>Financial Conduct Authority</t>
+        </is>
+      </c>
+      <c r="D22" s="102" t="inlineStr">
+        <is>
+          <t>Regulator</t>
+        </is>
+      </c>
+      <c r="E22" s="102" t="inlineStr">
+        <is>
+          <t>Whether any FCA Handbook page, Market Watch, or Technical Note addresses how a reasonable adjustment (interpreter/captioner/AI note-taker) is handled when the employee or meeting sits under a Chinese Wall (SYSC 10.2) or insider list (UK MAR Art. 18); if none, is anything in draft.</t>
+        </is>
+      </c>
+      <c r="F22" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G22" s="114" t="n"/>
       <c r="H22" s="115">
         <f>IF(G22="","",WORKDAY(G22,20,$U$5:$U$28))</f>
@@ -5934,8 +5974,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R22" s="102" t="n"/>
-      <c r="S22" s="112" t="n"/>
+      <c r="R22" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:54 (Chinese Walls batch). Do not FOI named commercial banks — not FOIA bodies.</t>
+        </is>
+      </c>
+      <c r="S22" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U22" s="117" t="n">
         <v>46472</v>
       </c>
@@ -5945,10 +5993,26 @@
         <v>19</v>
       </c>
       <c r="B23" s="102" t="n"/>
-      <c r="C23" s="102" t="n"/>
-      <c r="D23" s="102" t="n"/>
-      <c r="E23" s="102" t="n"/>
-      <c r="F23" s="102" t="n"/>
+      <c r="C23" s="102" t="inlineStr">
+        <is>
+          <t>Financial Conduct Authority / Bank of England (as employers)</t>
+        </is>
+      </c>
+      <c r="D23" s="102" t="inlineStr">
+        <is>
+          <t>Regulator (employer capacity)</t>
+        </is>
+      </c>
+      <c r="E23" s="102" t="inlineStr">
+        <is>
+          <t>Whether a written process exists for adding a communication-support professional to a restricted-information meeting involving own staff, including insider-list inclusion and written acknowledgement.</t>
+        </is>
+      </c>
+      <c r="F23" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G23" s="114" t="n"/>
       <c r="H23" s="115">
         <f>IF(G23="","",WORKDAY(G23,20,$U$5:$U$28))</f>
@@ -5978,8 +6042,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R23" s="102" t="n"/>
-      <c r="S23" s="112" t="n"/>
+      <c r="R23" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:54 companion ask, same batch — employer-capacity letter, separate from the regulator-capacity one above.</t>
+        </is>
+      </c>
+      <c r="S23" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U23" s="117" t="n">
         <v>46475</v>
       </c>
@@ -5989,10 +6061,26 @@
         <v>20</v>
       </c>
       <c r="B24" s="102" t="n"/>
-      <c r="C24" s="102" t="n"/>
-      <c r="D24" s="102" t="n"/>
-      <c r="E24" s="102" t="n"/>
-      <c r="F24" s="102" t="n"/>
+      <c r="C24" s="102" t="inlineStr">
+        <is>
+          <t>Department for Work and Pensions (Access to Work)</t>
+        </is>
+      </c>
+      <c r="D24" s="102" t="inlineStr">
+        <is>
+          <t>DWP</t>
+        </is>
+      </c>
+      <c r="E24" s="102" t="inlineStr">
+        <is>
+          <t>Whether case-manager AtW staff guidance (not the public employer factsheet) includes a TUPE carry-forward provision, and how many TUPE-transfer cases in the last 24 months used it, split by transfer direction (public-to-private / private-to-public / private-to-private).</t>
+        </is>
+      </c>
+      <c r="F24" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G24" s="114" t="n"/>
       <c r="H24" s="115">
         <f>IF(G24="","",WORKDAY(G24,20,$U$5:$U$28))</f>
@@ -6022,8 +6110,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R24" s="102" t="n"/>
-      <c r="S24" s="112" t="n"/>
+      <c r="R24" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:55 (TUPE batch).</t>
+        </is>
+      </c>
+      <c r="S24" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U24" s="117" t="n">
         <v>46510</v>
       </c>
@@ -6033,10 +6129,26 @@
         <v>21</v>
       </c>
       <c r="B25" s="102" t="n"/>
-      <c r="C25" s="102" t="n"/>
-      <c r="D25" s="102" t="n"/>
-      <c r="E25" s="102" t="n"/>
-      <c r="F25" s="102" t="n"/>
+      <c r="C25" s="102" t="inlineStr">
+        <is>
+          <t>SWL local authorities + SWL ICB (six-borough ask)</t>
+        </is>
+      </c>
+      <c r="D25" s="102" t="inlineStr">
+        <is>
+          <t>Council / ICB</t>
+        </is>
+      </c>
+      <c r="E25" s="102" t="inlineStr">
+        <is>
+          <t>For outsourced/TUPE-transferred services (interpreting, care, facilities, IT), whether the contract specifies continuity of any existing BSL/communication-support arrangement, and whether any TUPE transfer in the last 3 years caused a recorded gap in interpreter provision.</t>
+        </is>
+      </c>
+      <c r="F25" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G25" s="114" t="n"/>
       <c r="H25" s="115">
         <f>IF(G25="","",WORKDAY(G25,20,$U$5:$U$28))</f>
@@ -6066,8 +6178,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R25" s="102" t="n"/>
-      <c r="S25" s="112" t="n"/>
+      <c r="R25" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:56 (TUPE + outsourced-services batches).</t>
+        </is>
+      </c>
+      <c r="S25" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U25" s="117" t="n">
         <v>46538</v>
       </c>
@@ -6077,10 +6197,26 @@
         <v>22</v>
       </c>
       <c r="B26" s="102" t="n"/>
-      <c r="C26" s="102" t="n"/>
-      <c r="D26" s="102" t="n"/>
-      <c r="E26" s="102" t="n"/>
-      <c r="F26" s="102" t="n"/>
+      <c r="C26" s="102" t="inlineStr">
+        <is>
+          <t>Named SWL/SEL employing bodies (one letter per body)</t>
+        </is>
+      </c>
+      <c r="D26" s="102" t="inlineStr">
+        <is>
+          <t>Employer body</t>
+        </is>
+      </c>
+      <c r="E26" s="102" t="inlineStr">
+        <is>
+          <t>Yes/no/number only: does the current staff IT-support, payroll/HR shared-service, facilities helpdesk, whistleblowing/ethics line, and pension/benefits helpline each specify a non-voice contact channel, and who pays if a Deaf employee needs an interpreter or VRS minute to use it.</t>
+        </is>
+      </c>
+      <c r="F26" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G26" s="114" t="n"/>
       <c r="H26" s="115">
         <f>IF(G26="","",WORKDAY(G26,20,$U$5:$U$28))</f>
@@ -6110,8 +6246,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R26" s="102" t="n"/>
-      <c r="S26" s="112" t="n"/>
+      <c r="R26" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:57 (outsourced-services + SLA/HR-IT batches).</t>
+        </is>
+      </c>
+      <c r="S26" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U26" s="117" t="n">
         <v>46629</v>
       </c>
@@ -6121,10 +6265,26 @@
         <v>23</v>
       </c>
       <c r="B27" s="102" t="n"/>
-      <c r="C27" s="102" t="n"/>
-      <c r="D27" s="102" t="n"/>
-      <c r="E27" s="102" t="n"/>
-      <c r="F27" s="102" t="n"/>
+      <c r="C27" s="102" t="inlineStr">
+        <is>
+          <t>Named SWL/SEL employing bodies (one letter per body)</t>
+        </is>
+      </c>
+      <c r="D27" s="102" t="inlineStr">
+        <is>
+          <t>Employer body</t>
+        </is>
+      </c>
+      <c r="E27" s="102" t="inlineStr">
+        <is>
+          <t>For the same helplines, split by contract type (substantive staff vs agency/bank/contractor): published SLA per queue if different, and median calendar days to fulfilment of a reasonable-adjustment/interpreter request.</t>
+        </is>
+      </c>
+      <c r="F27" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G27" s="114" t="n"/>
       <c r="H27" s="115">
         <f>IF(G27="","",WORKDAY(G27,20,$U$5:$U$28))</f>
@@ -6154,8 +6314,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R27" s="102" t="n"/>
-      <c r="S27" s="112" t="n"/>
+      <c r="R27" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:58 (SLA/HR-IT batch).</t>
+        </is>
+      </c>
+      <c r="S27" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U27" s="117" t="n">
         <v>46748</v>
       </c>
@@ -6165,10 +6333,26 @@
         <v>24</v>
       </c>
       <c r="B28" s="102" t="n"/>
-      <c r="C28" s="102" t="n"/>
-      <c r="D28" s="102" t="n"/>
-      <c r="E28" s="102" t="n"/>
-      <c r="F28" s="102" t="n"/>
+      <c r="C28" s="102" t="inlineStr">
+        <is>
+          <t>SWL local authorities + SWL ICB (six-borough ask)</t>
+        </is>
+      </c>
+      <c r="D28" s="102" t="inlineStr">
+        <is>
+          <t>Council / ICB</t>
+        </is>
+      </c>
+      <c r="E28" s="102" t="inlineStr">
+        <is>
+          <t>Whether the OH provider's PEEP template asks if an employee works alone/out of hours; count of vibrating/critical-alert pagers or visual-alarm devices issued to staff in last 12 months; whether a BSL interpreter is routinely offered for staff OH appointments and at whose cost.</t>
+        </is>
+      </c>
+      <c r="F28" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G28" s="114" t="n"/>
       <c r="H28" s="115">
         <f>IF(G28="","",WORKDAY(G28,20,$U$5:$U$28))</f>
@@ -6198,8 +6382,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R28" s="102" t="n"/>
-      <c r="S28" s="112" t="n"/>
+      <c r="R28" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:59 (OH-workplace batch).</t>
+        </is>
+      </c>
+      <c r="S28" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
       <c r="U28" s="117" t="n">
         <v>46749</v>
       </c>
@@ -6209,10 +6401,26 @@
         <v>25</v>
       </c>
       <c r="B29" s="102" t="n"/>
-      <c r="C29" s="102" t="n"/>
-      <c r="D29" s="102" t="n"/>
-      <c r="E29" s="102" t="n"/>
-      <c r="F29" s="102" t="n"/>
+      <c r="C29" s="102" t="inlineStr">
+        <is>
+          <t>Named SWL/SEL Trusts + the ICB</t>
+        </is>
+      </c>
+      <c r="D29" s="102" t="inlineStr">
+        <is>
+          <t>Trust / ICB</t>
+        </is>
+      </c>
+      <c r="E29" s="102" t="inlineStr">
+        <is>
+          <t>Last financial year: BSL interpreter bookings requested/fulfilled/cancelled; face-to-face vs VRI split; unit rate if held centrally.</t>
+        </is>
+      </c>
+      <c r="F29" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G29" s="114" t="n"/>
       <c r="H29" s="115">
         <f>IF(G29="","",WORKDAY(G29,20,$U$5:$U$28))</f>
@@ -6242,18 +6450,42 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R29" s="102" t="n"/>
-      <c r="S29" s="112" t="n"/>
+      <c r="R29" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:60 (interpreter-regulation batch) — fold into existing companion log.</t>
+        </is>
+      </c>
+      <c r="S29" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="21.75" customHeight="1" s="74">
       <c r="A30" s="111" t="n">
         <v>26</v>
       </c>
       <c r="B30" s="102" t="n"/>
-      <c r="C30" s="102" t="n"/>
-      <c r="D30" s="102" t="n"/>
-      <c r="E30" s="102" t="n"/>
-      <c r="F30" s="102" t="n"/>
+      <c r="C30" s="102" t="inlineStr">
+        <is>
+          <t>NRCPD (right of reply first — not a public authority)</t>
+        </is>
+      </c>
+      <c r="D30" s="102" t="inlineStr">
+        <is>
+          <t>Right of reply</t>
+        </is>
+      </c>
+      <c r="E30" s="102" t="inlineStr">
+        <is>
+          <t>Unique registrant count by category (RSLI/TSLI/Deaf-relay) and nation, and complaints received/closed with sanctions, 2023-25.</t>
+        </is>
+      </c>
+      <c r="F30" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G30" s="114" t="n"/>
       <c r="H30" s="115">
         <f>IF(G30="","",WORKDAY(G30,20,$U$5:$U$28))</f>
@@ -6283,18 +6515,42 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R30" s="102" t="n"/>
-      <c r="S30" s="112" t="n"/>
+      <c r="R30" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:61. NRCPD is not FOIA-bound — approach via right of reply, not a formal FOI request.</t>
+        </is>
+      </c>
+      <c r="S30" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="21.75" customHeight="1" s="74">
       <c r="A31" s="111" t="n">
         <v>27</v>
       </c>
       <c r="B31" s="102" t="n"/>
-      <c r="C31" s="102" t="n"/>
-      <c r="D31" s="102" t="n"/>
-      <c r="E31" s="102" t="n"/>
-      <c r="F31" s="102" t="n"/>
+      <c r="C31" s="102" t="inlineStr">
+        <is>
+          <t>Crown Commercial Service (or one participating ICB)</t>
+        </is>
+      </c>
+      <c r="D31" s="102" t="inlineStr">
+        <is>
+          <t>National body</t>
+        </is>
+      </c>
+      <c r="E31" s="102" t="inlineStr">
+        <is>
+          <t>Under the RM6302 (or successor) interpreting framework Lot, whether a BSL-specific fulfilment KPI exists separate from the general interpreting KPI, and performance against it last financial year.</t>
+        </is>
+      </c>
+      <c r="F31" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G31" s="114" t="n"/>
       <c r="H31" s="115">
         <f>IF(G31="","",WORKDAY(G31,20,$U$5:$U$28))</f>
@@ -6324,18 +6580,42 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R31" s="102" t="n"/>
-      <c r="S31" s="112" t="n"/>
+      <c r="R31" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:62 (interpreter-regulation batch).</t>
+        </is>
+      </c>
+      <c r="S31" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="21.75" customHeight="1" s="74">
       <c r="A32" s="111" t="n">
         <v>28</v>
       </c>
       <c r="B32" s="102" t="n"/>
-      <c r="C32" s="102" t="n"/>
-      <c r="D32" s="102" t="n"/>
-      <c r="E32" s="102" t="n"/>
-      <c r="F32" s="102" t="n"/>
+      <c r="C32" s="102" t="inlineStr">
+        <is>
+          <t>SWL/SEL ICBs and mental-health trusts</t>
+        </is>
+      </c>
+      <c r="D32" s="102" t="inlineStr">
+        <is>
+          <t>ICB / Trust</t>
+        </is>
+      </c>
+      <c r="E32" s="102" t="inlineStr">
+        <is>
+          <t>Whether an adult autism and/or ADHD assessment pathway with a BSL-fluent clinician, or a contracted interpreter for the full assessment, is offered as standard, and completed-assessment count for a Deaf/BSL-using adult, last 24 months.</t>
+        </is>
+      </c>
+      <c r="F32" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G32" s="114" t="n"/>
       <c r="H32" s="115">
         <f>IF(G32="","",WORKDAY(G32,20,$U$5:$U$28))</f>
@@ -6365,18 +6645,42 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R32" s="102" t="n"/>
-      <c r="S32" s="112" t="n"/>
+      <c r="R32" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:63 (neurodivergence batch).</t>
+        </is>
+      </c>
+      <c r="S32" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="21.75" customHeight="1" s="74">
       <c r="A33" s="111" t="n">
         <v>29</v>
       </c>
       <c r="B33" s="102" t="n"/>
-      <c r="C33" s="102" t="n"/>
-      <c r="D33" s="102" t="n"/>
-      <c r="E33" s="102" t="n"/>
-      <c r="F33" s="102" t="n"/>
+      <c r="C33" s="102" t="inlineStr">
+        <is>
+          <t>SWL local authorities (six-borough ask)</t>
+        </is>
+      </c>
+      <c r="D33" s="102" t="inlineStr">
+        <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="E33" s="102" t="inlineStr">
+        <is>
+          <t>Number of EHCPs in the last 3 years recording deafness alongside autism or ADHD as a co-occurring need, and whether the EHCP template has a discrete dual-need field.</t>
+        </is>
+      </c>
+      <c r="F33" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G33" s="114" t="n"/>
       <c r="H33" s="115">
         <f>IF(G33="","",WORKDAY(G33,20,$U$5:$U$28))</f>
@@ -6406,18 +6710,42 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R33" s="102" t="n"/>
-      <c r="S33" s="112" t="n"/>
+      <c r="R33" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:64 (neurodivergence batch).</t>
+        </is>
+      </c>
+      <c r="S33" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="21.75" customHeight="1" s="74">
       <c r="A34" s="111" t="n">
         <v>30</v>
       </c>
       <c r="B34" s="102" t="n"/>
-      <c r="C34" s="102" t="n"/>
-      <c r="D34" s="102" t="n"/>
-      <c r="E34" s="102" t="n"/>
-      <c r="F34" s="102" t="n"/>
+      <c r="C34" s="102" t="inlineStr">
+        <is>
+          <t>DfE / NDCS / BATOD (right of reply first)</t>
+        </is>
+      </c>
+      <c r="D34" s="102" t="inlineStr">
+        <is>
+          <t>Right of reply</t>
+        </is>
+      </c>
+      <c r="E34" s="102" t="inlineStr">
+        <is>
+          <t>Whether parental hearing status has ever been a CRIDE survey or DfE School Census question; if not, whether it was ever proposed and rejected, and why.</t>
+        </is>
+      </c>
+      <c r="F34" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G34" s="114" t="n"/>
       <c r="H34" s="115">
         <f>IF(G34="","",WORKDAY(G34,20,$U$5:$U$28))</f>
@@ -6447,18 +6775,42 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R34" s="102" t="n"/>
-      <c r="S34" s="112" t="n"/>
+      <c r="R34" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:65 (CODA batch) — approach via right of reply before any formal FOI.</t>
+        </is>
+      </c>
+      <c r="S34" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="21.75" customHeight="1" s="74">
       <c r="A35" s="111" t="n">
         <v>31</v>
       </c>
       <c r="B35" s="102" t="n"/>
-      <c r="C35" s="102" t="n"/>
-      <c r="D35" s="102" t="n"/>
-      <c r="E35" s="102" t="n"/>
-      <c r="F35" s="102" t="n"/>
+      <c r="C35" s="102" t="inlineStr">
+        <is>
+          <t>SWL local authorities (six-borough ask)</t>
+        </is>
+      </c>
+      <c r="D35" s="102" t="inlineStr">
+        <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="E35" s="102" t="inlineStr">
+        <is>
+          <t>Number of young-carer assessments in the last 3 years citing interpreting/communication support for a Deaf/BSL-using parent, and whether the assessment template has a discrete field for this.</t>
+        </is>
+      </c>
+      <c r="F35" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G35" s="114" t="n"/>
       <c r="H35" s="115">
         <f>IF(G35="","",WORKDAY(G35,20,$U$5:$U$28))</f>
@@ -6488,18 +6840,42 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R35" s="102" t="n"/>
-      <c r="S35" s="112" t="n"/>
+      <c r="R35" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:66 (CODA batch).</t>
+        </is>
+      </c>
+      <c r="S35" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="21.75" customHeight="1" s="74">
       <c r="A36" s="111" t="n">
         <v>32</v>
       </c>
       <c r="B36" s="102" t="n"/>
-      <c r="C36" s="102" t="n"/>
-      <c r="D36" s="102" t="n"/>
-      <c r="E36" s="102" t="n"/>
-      <c r="F36" s="102" t="n"/>
+      <c r="C36" s="102" t="inlineStr">
+        <is>
+          <t>SWL local authorities (six-borough ask)</t>
+        </is>
+      </c>
+      <c r="D36" s="102" t="inlineStr">
+        <is>
+          <t>Council</t>
+        </is>
+      </c>
+      <c r="E36" s="102" t="inlineStr">
+        <is>
+          <t>For social-care needs assessments and Freedom Pass/concessionary-travel applications from people aged 65+, whether Deaf/BSL communication need is recorded as a discrete flag distinct from general hearing loss, and how many such flagged records exist.</t>
+        </is>
+      </c>
+      <c r="F36" s="102" t="inlineStr">
+        <is>
+          <t>Not sent</t>
+        </is>
+      </c>
       <c r="G36" s="114" t="n"/>
       <c r="H36" s="115">
         <f>IF(G36="","",WORKDAY(G36,20,$U$5:$U$28))</f>
@@ -6529,8 +6905,16 @@
           <t>No</t>
         </is>
       </c>
-      <c r="R36" s="102" t="n"/>
-      <c r="S36" s="112" t="n"/>
+      <c r="R36" s="102" t="inlineStr">
+        <is>
+          <t>Dossier FOI n:67 (Elderly Deaf batch).</t>
+        </is>
+      </c>
+      <c r="S36" s="112" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="21.75" customHeight="1" s="74">
       <c r="A37" s="111" t="n">

</xml_diff>